<commit_message>
fix: ret/call fix, and new error
-ret and call has been fixed

-new error happens when stack instruction and ret/call is used closely
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F95EC0-0714-4198-BBC8-65B874E0F001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="4290" yWindow="2580" windowWidth="28800" windowHeight="11295" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -944,12 +944,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -960,6 +954,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1308,54 +1308,54 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="8" t="s">
@@ -1599,18 +1599,18 @@
         <v>gen[4]</v>
       </c>
       <c r="O15" s="8"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="11"/>
-      <c r="W15" s="11"/>
-      <c r="X15" s="11"/>
-      <c r="Y15" s="11"/>
-      <c r="Z15" s="11"/>
-      <c r="AA15" s="11"/>
-      <c r="AB15" s="11"/>
-      <c r="AC15" s="11"/>
-      <c r="AD15" s="11"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="11"/>
+      <c r="U15" s="9"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9"/>
+      <c r="Z15" s="9"/>
+      <c r="AA15" s="9"/>
+      <c r="AB15" s="9"/>
+      <c r="AC15" s="9"/>
+      <c r="AD15" s="9"/>
+      <c r="AF15" s="9"/>
+      <c r="AG15" s="9"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
@@ -2324,12 +2324,12 @@
       <c r="R34" t="s">
         <v>181</v>
       </c>
-      <c r="T34" s="11"/>
-      <c r="U34" s="11"/>
-      <c r="V34" s="11"/>
-      <c r="W34" s="11"/>
-      <c r="X34" s="11"/>
-      <c r="Y34" s="11"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
@@ -2367,12 +2367,12 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8"/>
-      <c r="T35" s="11"/>
-      <c r="U35" s="11"/>
-      <c r="V35" s="11"/>
-      <c r="W35" s="11"/>
-      <c r="X35" s="11"/>
-      <c r="Y35" s="11"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
@@ -2532,16 +2532,16 @@
       <c r="E40" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="F40" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="12" t="s">
+      <c r="G40" s="11"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="J40" s="13"/>
-      <c r="K40" s="14"/>
+      <c r="J40" s="11"/>
+      <c r="K40" s="12"/>
       <c r="L40" s="5" t="s">
         <v>141</v>
       </c>
@@ -3622,6 +3622,165 @@
     </row>
   </sheetData>
   <mergeCells count="183">
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="L62:O62"/>
+    <mergeCell ref="L68:O68"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N56:O56"/>
+    <mergeCell ref="N57:O57"/>
+    <mergeCell ref="N58:O58"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="N55:O55"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="L11:L35"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="C63:C69"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="G55:H55"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="I64:K64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="I65:K65"/>
+    <mergeCell ref="G68:H68"/>
     <mergeCell ref="C37:C39"/>
     <mergeCell ref="I35:K35"/>
     <mergeCell ref="I36:K36"/>
@@ -3646,165 +3805,6 @@
     <mergeCell ref="I62:K62"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="F49:H49"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="I65:K65"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="C63:C69"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="L11:L35"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="L62:O62"/>
-    <mergeCell ref="L68:O68"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N56:O56"/>
-    <mergeCell ref="N57:O57"/>
-    <mergeCell ref="N58:O58"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="N55:O55"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="N60:O60"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: fix branch commit issue, abother store issue detected
-fixed commit error happening after missed branch prediction

-still, there is a store and load issue going on
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -944,6 +944,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -954,12 +960,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1308,54 +1308,54 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="8" t="s">
@@ -1599,18 +1599,18 @@
         <v>gen[4]</v>
       </c>
       <c r="O15" s="8"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
-      <c r="Y15" s="9"/>
-      <c r="Z15" s="9"/>
-      <c r="AA15" s="9"/>
-      <c r="AB15" s="9"/>
-      <c r="AC15" s="9"/>
-      <c r="AD15" s="9"/>
-      <c r="AF15" s="9"/>
-      <c r="AG15" s="9"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="11"/>
+      <c r="AA15" s="11"/>
+      <c r="AB15" s="11"/>
+      <c r="AC15" s="11"/>
+      <c r="AD15" s="11"/>
+      <c r="AF15" s="11"/>
+      <c r="AG15" s="11"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
@@ -2324,12 +2324,12 @@
       <c r="R34" t="s">
         <v>181</v>
       </c>
-      <c r="T34" s="9"/>
-      <c r="U34" s="9"/>
-      <c r="V34" s="9"/>
-      <c r="W34" s="9"/>
-      <c r="X34" s="9"/>
-      <c r="Y34" s="9"/>
+      <c r="T34" s="11"/>
+      <c r="U34" s="11"/>
+      <c r="V34" s="11"/>
+      <c r="W34" s="11"/>
+      <c r="X34" s="11"/>
+      <c r="Y34" s="11"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
@@ -2367,12 +2367,12 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8"/>
-      <c r="T35" s="9"/>
-      <c r="U35" s="9"/>
-      <c r="V35" s="9"/>
-      <c r="W35" s="9"/>
-      <c r="X35" s="9"/>
-      <c r="Y35" s="9"/>
+      <c r="T35" s="11"/>
+      <c r="U35" s="11"/>
+      <c r="V35" s="11"/>
+      <c r="W35" s="11"/>
+      <c r="X35" s="11"/>
+      <c r="Y35" s="11"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
@@ -2532,16 +2532,16 @@
       <c r="E40" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="F40" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="G40" s="11"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="10" t="s">
+      <c r="G40" s="13"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="J40" s="11"/>
-      <c r="K40" s="12"/>
+      <c r="J40" s="13"/>
+      <c r="K40" s="14"/>
       <c r="L40" s="5" t="s">
         <v>141</v>
       </c>
@@ -3622,6 +3622,165 @@
     </row>
   </sheetData>
   <mergeCells count="183">
+    <mergeCell ref="L69:O69"/>
+    <mergeCell ref="L70:O70"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="C45:C50"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="C59:C62"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="I65:K65"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="I64:K64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="C63:C69"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="G55:H55"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="L11:L35"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
     <mergeCell ref="C41:C42"/>
     <mergeCell ref="N61:O61"/>
     <mergeCell ref="L62:O62"/>
@@ -3646,165 +3805,6 @@
     <mergeCell ref="I44:K44"/>
     <mergeCell ref="I43:K43"/>
     <mergeCell ref="C43:C44"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="L11:L35"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="C63:C69"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="I65:K65"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="L69:O69"/>
-    <mergeCell ref="L70:O70"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C45:C50"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="F61:H61"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="F49:H49"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: trying to fix some issue
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F95EC0-0714-4198-BBC8-65B874E0F001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD979BF7-DB29-4BCF-A17C-9F767B35A295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="2580" windowWidth="28800" windowHeight="11295" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="194">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -777,10 +777,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ALU exp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>sets</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -802,6 +798,18 @@
   </si>
   <si>
     <t>testi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flow exp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>block</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>blocks pipeline</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -944,12 +952,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -960,6 +962,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1308,54 +1316,54 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="8" t="s">
@@ -1599,18 +1607,18 @@
         <v>gen[4]</v>
       </c>
       <c r="O15" s="8"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="11"/>
-      <c r="W15" s="11"/>
-      <c r="X15" s="11"/>
-      <c r="Y15" s="11"/>
-      <c r="Z15" s="11"/>
-      <c r="AA15" s="11"/>
-      <c r="AB15" s="11"/>
-      <c r="AC15" s="11"/>
-      <c r="AD15" s="11"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="11"/>
+      <c r="U15" s="9"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9"/>
+      <c r="Z15" s="9"/>
+      <c r="AA15" s="9"/>
+      <c r="AB15" s="9"/>
+      <c r="AC15" s="9"/>
+      <c r="AD15" s="9"/>
+      <c r="AF15" s="9"/>
+      <c r="AG15" s="9"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
@@ -2297,7 +2305,7 @@
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>13</v>
@@ -2307,7 +2315,7 @@
       </c>
       <c r="H34" s="8"/>
       <c r="I34" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
@@ -2324,12 +2332,12 @@
       <c r="R34" t="s">
         <v>181</v>
       </c>
-      <c r="T34" s="11"/>
-      <c r="U34" s="11"/>
-      <c r="V34" s="11"/>
-      <c r="W34" s="11"/>
-      <c r="X34" s="11"/>
-      <c r="Y34" s="11"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
@@ -2367,12 +2375,12 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8"/>
-      <c r="T35" s="11"/>
-      <c r="U35" s="11"/>
-      <c r="V35" s="11"/>
-      <c r="W35" s="11"/>
-      <c r="X35" s="11"/>
-      <c r="Y35" s="11"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
@@ -2384,7 +2392,7 @@
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>13</v>
@@ -2394,7 +2402,7 @@
       </c>
       <c r="H36" s="8"/>
       <c r="I36" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
@@ -2458,7 +2466,7 @@
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
@@ -2468,7 +2476,7 @@
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
@@ -2522,26 +2530,26 @@
       <c r="B40" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>185</v>
+      <c r="C40" s="5" t="s">
+        <v>191</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F40" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="F40" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="J40" s="13"/>
-      <c r="K40" s="14"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="J40" s="11"/>
+      <c r="K40" s="12"/>
       <c r="L40" s="5" t="s">
         <v>141</v>
       </c>
@@ -3622,6 +3630,165 @@
     </row>
   </sheetData>
   <mergeCells count="183">
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="L62:O62"/>
+    <mergeCell ref="L68:O68"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N56:O56"/>
+    <mergeCell ref="N57:O57"/>
+    <mergeCell ref="N58:O58"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="N55:O55"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="L11:L35"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="G55:H55"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="I64:K64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="C63:C69"/>
+    <mergeCell ref="C57:C58"/>
     <mergeCell ref="L69:O69"/>
     <mergeCell ref="L70:O70"/>
     <mergeCell ref="C53:C54"/>
@@ -3646,165 +3813,6 @@
     <mergeCell ref="G65:H65"/>
     <mergeCell ref="I65:K65"/>
     <mergeCell ref="G68:H68"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="C63:C69"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="L11:L35"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="L62:O62"/>
-    <mergeCell ref="L68:O68"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N56:O56"/>
-    <mergeCell ref="N57:O57"/>
-    <mergeCell ref="N58:O58"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="N55:O55"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="N60:O60"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: alu problem fixed
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD979BF7-DB29-4BCF-A17C-9F767B35A295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF40D3A-E69F-4590-BFA5-97F916EE40D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="6420" yWindow="135" windowWidth="28800" windowHeight="12915" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -952,6 +952,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -962,12 +968,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1316,54 +1316,54 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="8" t="s">
@@ -1607,18 +1607,18 @@
         <v>gen[4]</v>
       </c>
       <c r="O15" s="8"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
-      <c r="Y15" s="9"/>
-      <c r="Z15" s="9"/>
-      <c r="AA15" s="9"/>
-      <c r="AB15" s="9"/>
-      <c r="AC15" s="9"/>
-      <c r="AD15" s="9"/>
-      <c r="AF15" s="9"/>
-      <c r="AG15" s="9"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="11"/>
+      <c r="AA15" s="11"/>
+      <c r="AB15" s="11"/>
+      <c r="AC15" s="11"/>
+      <c r="AD15" s="11"/>
+      <c r="AF15" s="11"/>
+      <c r="AG15" s="11"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
@@ -2332,12 +2332,12 @@
       <c r="R34" t="s">
         <v>181</v>
       </c>
-      <c r="T34" s="9"/>
-      <c r="U34" s="9"/>
-      <c r="V34" s="9"/>
-      <c r="W34" s="9"/>
-      <c r="X34" s="9"/>
-      <c r="Y34" s="9"/>
+      <c r="T34" s="11"/>
+      <c r="U34" s="11"/>
+      <c r="V34" s="11"/>
+      <c r="W34" s="11"/>
+      <c r="X34" s="11"/>
+      <c r="Y34" s="11"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
@@ -2375,12 +2375,12 @@
         <v>gen[24]</v>
       </c>
       <c r="O35" s="8"/>
-      <c r="T35" s="9"/>
-      <c r="U35" s="9"/>
-      <c r="V35" s="9"/>
-      <c r="W35" s="9"/>
-      <c r="X35" s="9"/>
-      <c r="Y35" s="9"/>
+      <c r="T35" s="11"/>
+      <c r="U35" s="11"/>
+      <c r="V35" s="11"/>
+      <c r="W35" s="11"/>
+      <c r="X35" s="11"/>
+      <c r="Y35" s="11"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
@@ -2540,16 +2540,16 @@
       <c r="E40" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="F40" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="G40" s="11"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="10" t="s">
+      <c r="G40" s="13"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="J40" s="11"/>
-      <c r="K40" s="12"/>
+      <c r="J40" s="13"/>
+      <c r="K40" s="14"/>
       <c r="L40" s="5" t="s">
         <v>141</v>
       </c>
@@ -3630,6 +3630,165 @@
     </row>
   </sheetData>
   <mergeCells count="183">
+    <mergeCell ref="L69:O69"/>
+    <mergeCell ref="L70:O70"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="C45:C50"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="C59:C62"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="I65:K65"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="I64:K64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="C63:C69"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="G55:H55"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="L11:L35"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
     <mergeCell ref="C41:C42"/>
     <mergeCell ref="N61:O61"/>
     <mergeCell ref="L62:O62"/>
@@ -3654,165 +3813,6 @@
     <mergeCell ref="I44:K44"/>
     <mergeCell ref="I43:K43"/>
     <mergeCell ref="C43:C44"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="L11:L35"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="C63:C69"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="L69:O69"/>
-    <mergeCell ref="L70:O70"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C45:C50"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="F61:H61"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="I65:K65"/>
-    <mergeCell ref="G68:H68"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: call with base, interrupt being implimented
-call can now jump to register base + immidate

-interrupt sequence being implimented
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF40D3A-E69F-4590-BFA5-97F916EE40D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B9BC80-A643-41C5-AC3C-1B0626FFB847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="135" windowWidth="28800" windowHeight="12915" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="201">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -161,10 +161,6 @@
     <t/>
   </si>
   <si>
-    <t>mode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>8L</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -197,14 +193,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>mmub</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>mmul</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>dma</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -245,14 +233,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>baseA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>baseB</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -381,14 +361,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>mmu base = base + offset</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>mmu limit = base + offset</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>dma srcL = base + offset</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -417,10 +389,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>int vec[baseB + imm] = baseA</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>dest = stack.pop()</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -489,26 +457,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>exp2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>level</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>modevec</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0~255</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>mode vec = base + off</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>iret</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -810,6 +762,82 @@
   </si>
   <si>
     <t>blocks pipeline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ABI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>return</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arg1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>callee</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>caller</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>addr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>stistack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ldistack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>interpri</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>istack = src</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dest = istack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>m(0~255)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sbase</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lbase</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>invalTLB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int_vec[id] = base + imm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int_pri[id] = imm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>d(0~63)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>m(0~15)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -858,7 +886,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -918,13 +946,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -952,12 +1017,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -969,6 +1028,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1316,58 +1396,58 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
+      <c r="B6" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -1379,7 +1459,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
@@ -1387,48 +1467,50 @@
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
       <c r="L10" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="O10" s="8"/>
+        <v>49</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="O10" s="15" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>27</v>
@@ -1443,28 +1525,30 @@
         <v>13</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="8" t="s">
-        <v>139</v>
+      <c r="L11" s="16" t="s">
+        <v>127</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="8" t="str">
+      <c r="N11" s="15" t="str">
         <f t="shared" ref="N11:N16" si="0">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M11)),"]")</f>
         <v>gen[0]</v>
       </c>
-      <c r="O11" s="8"/>
+      <c r="O11" s="5" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="3" t="str">
@@ -1481,27 +1565,29 @@
         <v>13</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
+      <c r="L12" s="17"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
       </c>
-      <c r="N12" s="8" t="str">
+      <c r="N12" s="15" t="str">
         <f t="shared" si="0"/>
         <v>gen[1]</v>
       </c>
-      <c r="O12" s="8"/>
+      <c r="O12" s="16" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="3" t="str">
@@ -1515,28 +1601,28 @@
         <v>12</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="8" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
+      <c r="L13" s="17"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
       </c>
-      <c r="N13" s="8" t="str">
+      <c r="N13" s="15" t="str">
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="8"/>
+      <c r="O13" s="17"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="3" t="str">
@@ -1553,27 +1639,27 @@
         <v>13</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
+      <c r="L14" s="17"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
       </c>
-      <c r="N14" s="8" t="str">
+      <c r="N14" s="15" t="str">
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="8"/>
+      <c r="O14" s="17"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="3" t="str">
@@ -1590,39 +1676,39 @@
         <v>13</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
+      <c r="L15" s="17"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
       </c>
-      <c r="N15" s="8" t="str">
+      <c r="N15" s="15" t="str">
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="8"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="11"/>
-      <c r="W15" s="11"/>
-      <c r="X15" s="11"/>
-      <c r="Y15" s="11"/>
-      <c r="Z15" s="11"/>
-      <c r="AA15" s="11"/>
-      <c r="AB15" s="11"/>
-      <c r="AC15" s="11"/>
-      <c r="AD15" s="11"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="11"/>
+      <c r="O15" s="18"/>
+      <c r="U15" s="9"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9"/>
+      <c r="Z15" s="9"/>
+      <c r="AA15" s="9"/>
+      <c r="AB15" s="9"/>
+      <c r="AC15" s="9"/>
+      <c r="AD15" s="9"/>
+      <c r="AF15" s="9"/>
+      <c r="AG15" s="9"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="3" t="str">
@@ -1636,24 +1722,26 @@
         <v>12</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
+      <c r="L16" s="17"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
       </c>
-      <c r="N16" s="8" t="str">
+      <c r="N16" s="15" t="str">
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="8"/>
+      <c r="O16" s="16" t="s">
+        <v>185</v>
+      </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
@@ -1670,7 +1758,7 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="3" t="str">
@@ -1687,27 +1775,27 @@
         <v>13</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
+      <c r="L17" s="17"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
       </c>
-      <c r="N17" s="8" t="str">
+      <c r="N17" s="15" t="str">
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="8"/>
+      <c r="O17" s="17"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="3" t="str">
@@ -1715,35 +1803,35 @@
         <v>07</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H18" s="8"/>
       <c r="I18" s="8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
+      <c r="L18" s="17"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
       </c>
-      <c r="N18" s="8" t="str">
+      <c r="N18" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="8"/>
+      <c r="O18" s="17"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="3" t="str">
@@ -1760,28 +1848,28 @@
         <v>13</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
+      <c r="L19" s="17"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
       </c>
-      <c r="N19" s="8" t="str">
+      <c r="N19" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="8"/>
+      <c r="O19" s="17"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="3" t="str">
@@ -1789,36 +1877,36 @@
         <v>09</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="8" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
+      <c r="L20" s="17"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
       </c>
-      <c r="N20" s="8" t="str">
+      <c r="N20" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="8"/>
+      <c r="O20" s="17"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C21" s="8"/>
       <c r="D21" s="3" t="str">
@@ -1835,27 +1923,27 @@
         <v>13</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
+      <c r="L21" s="17"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
       </c>
-      <c r="N21" s="8" t="str">
+      <c r="N21" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="8"/>
+      <c r="O21" s="17"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" s="3" t="str">
@@ -1863,30 +1951,30 @@
         <v>0B</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="8" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
+      <c r="L22" s="17"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
       </c>
-      <c r="N22" s="8" t="str">
+      <c r="N22" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="8"/>
+      <c r="O22" s="17"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -1894,7 +1982,7 @@
     </row>
     <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="3" t="str">
@@ -1902,7 +1990,7 @@
         <v>0C</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>12</v>
@@ -1911,23 +1999,23 @@
         <v>13</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
+      <c r="L23" s="17"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
       </c>
-      <c r="N23" s="8" t="str">
+      <c r="N23" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="8"/>
+      <c r="O23" s="18"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -1935,7 +2023,7 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="3" t="str">
@@ -1943,34 +2031,36 @@
         <v>0D</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H24" s="8"/>
       <c r="I24" s="8" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
+      <c r="L24" s="17"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
       </c>
-      <c r="N24" s="8" t="str">
+      <c r="N24" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="8"/>
+      <c r="O24" s="16" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" s="3" t="str">
@@ -1978,7 +2068,7 @@
         <v>0E</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>12</v>
@@ -1987,27 +2077,27 @@
         <v>13</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
+      <c r="L25" s="17"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
       </c>
-      <c r="N25" s="8" t="str">
+      <c r="N25" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="8"/>
+      <c r="O25" s="17"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="3" t="str">
@@ -2015,34 +2105,34 @@
         <v>0F</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H26" s="8"/>
       <c r="I26" s="8" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
+      <c r="L26" s="17"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
       </c>
-      <c r="N26" s="8" t="str">
+      <c r="N26" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="8"/>
+      <c r="O26" s="17"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C27" s="8"/>
       <c r="D27" s="3" t="str">
@@ -2050,7 +2140,7 @@
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>12</v>
@@ -2059,27 +2149,27 @@
         <v>13</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
+      <c r="L27" s="17"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N27" s="8" t="str">
+      <c r="N27" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="8"/>
+      <c r="O27" s="17"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="3" t="str">
@@ -2087,7 +2177,7 @@
         <v>11</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>12</v>
@@ -2096,27 +2186,27 @@
         <v>13</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
+      <c r="L28" s="17"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="N28" s="8" t="str">
+      <c r="N28" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="8"/>
+      <c r="O28" s="17"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C29" s="8"/>
       <c r="D29" s="3" t="str">
@@ -2124,34 +2214,34 @@
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H29" s="8"/>
       <c r="I29" s="8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
+      <c r="L29" s="17"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="N29" s="8" t="str">
+      <c r="N29" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="8"/>
+      <c r="O29" s="17"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="3" t="str">
@@ -2159,7 +2249,7 @@
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>12</v>
@@ -2168,27 +2258,27 @@
         <v>13</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
+      <c r="L30" s="17"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="N30" s="8" t="str">
+      <c r="N30" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="8"/>
+      <c r="O30" s="17"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="3" t="str">
@@ -2196,7 +2286,7 @@
         <v>14</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>12</v>
@@ -2205,27 +2295,27 @@
         <v>13</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
+      <c r="L31" s="17"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="N31" s="8" t="str">
+      <c r="N31" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="8"/>
+      <c r="O31" s="18"/>
     </row>
     <row r="32" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="3" t="str">
@@ -2233,34 +2323,36 @@
         <v>15</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H32" s="8"/>
       <c r="I32" s="8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
+      <c r="L32" s="17"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="N32" s="8" t="str">
+      <c r="N32" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[21]</v>
       </c>
-      <c r="O32" s="8"/>
+      <c r="O32" s="16" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="3" t="str">
@@ -2268,36 +2360,36 @@
         <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
+      <c r="L33" s="17"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="N33" s="8" t="str">
+      <c r="N33" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="8"/>
+      <c r="O33" s="17"/>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="3" t="str">
@@ -2305,43 +2397,43 @@
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H34" s="8"/>
       <c r="I34" s="8" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
+      <c r="L34" s="17"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="N34" s="8" t="str">
+      <c r="N34" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="8"/>
+      <c r="O34" s="17"/>
       <c r="R34" t="s">
-        <v>181</v>
-      </c>
-      <c r="T34" s="11"/>
-      <c r="U34" s="11"/>
-      <c r="V34" s="11"/>
-      <c r="W34" s="11"/>
-      <c r="X34" s="11"/>
-      <c r="Y34" s="11"/>
+        <v>169</v>
+      </c>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="3" t="str">
@@ -2349,42 +2441,42 @@
         <v>18</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
+      <c r="L35" s="18"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="N35" s="8" t="str">
+      <c r="N35" s="15" t="str">
         <f t="shared" si="3"/>
         <v>gen[24]</v>
       </c>
-      <c r="O35" s="8"/>
-      <c r="T35" s="11"/>
-      <c r="U35" s="11"/>
-      <c r="V35" s="11"/>
-      <c r="W35" s="11"/>
-      <c r="X35" s="11"/>
-      <c r="Y35" s="11"/>
+      <c r="O35" s="18"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="3" t="str">
@@ -2392,38 +2484,40 @@
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H36" s="8"/>
       <c r="I36" s="8" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
       <c r="L36" s="5" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="N36" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="O36" s="8"/>
+      <c r="N36" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="O36" s="5" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D37" s="3" t="str">
         <f t="shared" ref="D37:D42" si="4">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D36)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D36)+1))</f>
@@ -2436,29 +2530,31 @@
         <v>12</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H37" s="8"/>
       <c r="I37" s="8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
       <c r="L37" s="8" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="M37" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1A</v>
       </c>
-      <c r="N37" s="8" t="s">
+      <c r="N37" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="O37" s="8"/>
+      <c r="O37" s="16" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="3" t="str">
@@ -2466,17 +2562,17 @@
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="8" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
@@ -2485,14 +2581,14 @@
         <f t="shared" si="2"/>
         <v>1B</v>
       </c>
-      <c r="N38" s="8" t="s">
+      <c r="N38" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="O38" s="8"/>
+      <c r="O38" s="17"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="3" t="str">
@@ -2509,10 +2605,10 @@
         <v>13</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
@@ -2521,50 +2617,52 @@
         <f t="shared" si="2"/>
         <v>1C</v>
       </c>
-      <c r="N39" s="8" t="s">
+      <c r="N39" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="O39" s="8"/>
+      <c r="O39" s="18"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="J40" s="13"/>
-      <c r="K40" s="14"/>
+        <v>180</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="G40" s="11"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="J40" s="11"/>
+      <c r="K40" s="12"/>
       <c r="L40" s="5" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="M40" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1D</v>
       </c>
-      <c r="N40" s="8" t="s">
+      <c r="N40" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="8"/>
+      <c r="O40" s="5" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>3</v>
@@ -2580,30 +2678,32 @@
         <v>12</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="H41" s="8"/>
       <c r="I41" s="8" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="5" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="M41" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1E</v>
       </c>
-      <c r="N41" s="8" t="s">
+      <c r="N41" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="O41" s="8"/>
+      <c r="O41" s="5" t="s">
+        <v>3</v>
+      </c>
       <c r="T41" s="2"/>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C42" s="8"/>
       <c r="D42" s="3" t="str">
@@ -2617,49 +2717,51 @@
         <v>13</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="H42" s="8"/>
       <c r="I42" s="8" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
       <c r="L42" s="5" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="M42" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1F</v>
       </c>
-      <c r="N42" s="8" t="s">
+      <c r="N42" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="8"/>
+      <c r="O42" s="5" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D43" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D42) + 1),"~",DEC2HEX(HEX2DEC(D42) + 32))</f>
         <v>20~3F</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H43" s="8"/>
       <c r="I43" s="8" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
@@ -2672,7 +2774,7 @@
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="3" t="str">
@@ -2680,59 +2782,59 @@
         <v>40~5F</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H44" s="8"/>
       <c r="I44" s="8" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
       <c r="L44" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="N44" s="8" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="O44" s="8"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D45" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D44,LEN(D44)-FIND("~",D44,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D44,LEN(D44)-FIND("~",D44,1))) + 8))</f>
         <v>60~67</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H45" s="8"/>
       <c r="I45" s="8" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
       <c r="L45" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>27</v>
@@ -2744,7 +2846,7 @@
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C46" s="8"/>
       <c r="D46" s="3" t="str">
@@ -2752,22 +2854,22 @@
         <v>68~6F</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H46" s="8"/>
       <c r="I46" s="8" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
       <c r="L46" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M46" s="3" t="str">
         <f t="shared" ref="M46:M59" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M45)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M45)+1))</f>
@@ -2780,7 +2882,7 @@
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C47" s="8"/>
       <c r="D47" s="4" t="str">
@@ -2788,22 +2890,22 @@
         <v>70</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H47" s="8"/>
       <c r="I47" s="8" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
       <c r="L47" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M47" s="3" t="str">
         <f t="shared" si="5"/>
@@ -2816,7 +2918,7 @@
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="3" t="str">
@@ -2824,33 +2926,33 @@
         <v>71</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
       <c r="L48" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M48" s="3" t="str">
         <f t="shared" si="5"/>
         <v>03</v>
       </c>
       <c r="N48" s="8" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="O48" s="8"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C49" s="8"/>
       <c r="D49" s="3" t="str">
@@ -2858,33 +2960,33 @@
         <v>72</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
       <c r="I49" s="8" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
       <c r="L49" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>04</v>
       </c>
       <c r="N49" s="8" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="O49" s="8"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C50" s="8"/>
       <c r="D50" s="3" t="str">
@@ -2892,58 +2994,56 @@
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
       <c r="L50" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>05</v>
       </c>
       <c r="N50" s="8" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="O50" s="8"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="6"/>
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F51" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G51" s="8" t="s">
-        <v>38</v>
-      </c>
+      <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
       <c r="L51" s="5" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="M51" s="3" t="str">
         <f t="shared" si="5"/>
@@ -2956,7 +3056,7 @@
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C52" s="8"/>
       <c r="D52" s="3" t="str">
@@ -2964,20 +3064,20 @@
         <v>75</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="8" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
       <c r="L52" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M52" s="3" t="str">
         <f t="shared" si="5"/>
@@ -2990,43 +3090,43 @@
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>65</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="C53" s="8"/>
       <c r="D53" s="3" t="str">
         <f t="shared" si="6"/>
         <v>76</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="F53" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="G53" s="8"/>
+        <v>188</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>115</v>
+      </c>
       <c r="H53" s="8"/>
       <c r="I53" s="8" t="s">
-        <v>119</v>
+        <v>191</v>
       </c>
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
       <c r="L53" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M53" s="3" t="str">
         <f t="shared" si="5"/>
         <v>08</v>
       </c>
       <c r="N53" s="8" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="O53" s="8"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C54" s="8"/>
       <c r="D54" s="3" t="str">
@@ -3034,204 +3134,202 @@
         <v>77</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>110</v>
+        <v>189</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="H54" s="4" t="s">
-        <v>116</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="G54" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="H54" s="8"/>
       <c r="I54" s="8" t="s">
-        <v>95</v>
+        <v>192</v>
       </c>
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
       <c r="L54" s="5" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="M54" s="3" t="str">
         <f t="shared" si="5"/>
         <v>09</v>
       </c>
       <c r="N54" s="8" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="O54" s="8"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C55" s="8" t="s">
-        <v>51</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="C55" s="8"/>
       <c r="D55" s="3" t="str">
-        <f t="shared" ref="D55:D70" si="7">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
+        <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>40</v>
+        <v>102</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G55" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H55" s="8"/>
+      <c r="G55" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="I55" s="8" t="s">
-        <v>86</v>
+        <v>197</v>
       </c>
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
       <c r="L55" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M55" s="3" t="str">
         <f t="shared" si="5"/>
         <v>0A</v>
       </c>
       <c r="N55" s="8" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="O55" s="8"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C56" s="8"/>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H56" s="8"/>
+        <v>190</v>
+      </c>
+      <c r="F56" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="H56" s="15" t="s">
+        <v>200</v>
+      </c>
       <c r="I56" s="8" t="s">
-        <v>87</v>
+        <v>198</v>
       </c>
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
       <c r="L56" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M56" s="3" t="str">
         <f t="shared" si="5"/>
         <v>0B</v>
       </c>
       <c r="N56" s="8" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="O56" s="8"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>108</v>
+        <v>48</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D56)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D56)+1))</f>
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>109</v>
+        <v>194</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
       <c r="I57" s="8" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
       <c r="L57" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M57" s="3" t="str">
         <f t="shared" si="5"/>
         <v>0C</v>
       </c>
       <c r="N57" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="O57" s="8"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C58" s="8"/>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>122</v>
+        <v>195</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
       <c r="I58" s="8" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="J58" s="8"/>
       <c r="K58" s="8"/>
       <c r="L58" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M58" s="3" t="str">
         <f t="shared" si="5"/>
         <v>0D</v>
       </c>
       <c r="N58" s="8" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="O58" s="8"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C59" s="8" t="s">
-        <v>113</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="C59" s="8"/>
       <c r="D59" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D59:D70" si="7">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D58)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D58)+1))</f>
         <v>7C</v>
       </c>
-      <c r="E59" s="3" t="s">
-        <v>111</v>
+      <c r="E59" s="19" t="s">
+        <v>196</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
       <c r="I59" s="8" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="J59" s="8"/>
       <c r="K59" s="8"/>
       <c r="L59" s="5" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="M59" s="3" t="str">
         <f t="shared" si="5"/>
@@ -3244,75 +3342,77 @@
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C60" s="8"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
       </c>
-      <c r="E60" s="3" t="s">
-        <v>111</v>
+      <c r="E60" s="19" t="s">
+        <v>103</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="8" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="J60" s="8"/>
       <c r="K60" s="8"/>
       <c r="L60" s="5" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="M60" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M59)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M59)+1))</f>
         <v>0F</v>
       </c>
       <c r="N60" s="8" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="O60" s="8"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C61" s="8"/>
+        <v>108</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>100</v>
+      </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7E</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
       <c r="I61" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J61" s="8"/>
       <c r="K61" s="8"/>
       <c r="L61" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M61" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,IF(HEX2DEC(M60) + 1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M60) + 1),"~",IF(HEX2DEC(M60) + 4 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M60) + 16))</f>
         <v>10~1F</v>
       </c>
       <c r="N61" s="8" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="O61" s="8"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C62" s="8"/>
       <c r="D62" s="3" t="str">
@@ -3320,10 +3420,10 @@
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
@@ -3333,7 +3433,7 @@
       <c r="J62" s="8"/>
       <c r="K62" s="8"/>
       <c r="L62" s="8" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="M62" s="8"/>
       <c r="N62" s="8"/>
@@ -3341,46 +3441,46 @@
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D63" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D62)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D62)+1))</f>
         <v>80</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H63" s="8"/>
       <c r="I63" s="8" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="J63" s="8"/>
       <c r="K63" s="8"/>
       <c r="L63" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="N63" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="O63" s="3" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C64" s="8"/>
       <c r="D64" s="3" t="str">
@@ -3388,22 +3488,22 @@
         <v>81</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H64" s="8"/>
       <c r="I64" s="8" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="J64" s="8"/>
       <c r="K64" s="8"/>
       <c r="L64" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="M64" s="7" t="s">
         <v>28</v>
@@ -3413,12 +3513,12 @@
         <v>4</v>
       </c>
       <c r="O64" s="4" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C65" s="8"/>
       <c r="D65" s="3" t="str">
@@ -3426,17 +3526,17 @@
         <v>82</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H65" s="8"/>
       <c r="I65" s="8" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
@@ -3452,12 +3552,12 @@
         <v>5</v>
       </c>
       <c r="O65" s="4" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C66" s="8"/>
       <c r="D66" s="3" t="str">
@@ -3465,17 +3565,17 @@
         <v>83</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G66" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H66" s="8"/>
       <c r="I66" s="8" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="J66" s="8"/>
       <c r="K66" s="8"/>
@@ -3484,19 +3584,19 @@
         <v>2</v>
       </c>
       <c r="M66" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N66" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(N65+1)</f>
         <v>6</v>
       </c>
       <c r="O66" s="4" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C67" s="8"/>
       <c r="D67" s="3" t="str">
@@ -3504,17 +3604,17 @@
         <v>84</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H67" s="8"/>
       <c r="I67" s="8" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="J67" s="8"/>
       <c r="K67" s="8"/>
@@ -3523,19 +3623,19 @@
         <v>3</v>
       </c>
       <c r="M67" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N67" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(N66+1)</f>
         <v>7</v>
       </c>
       <c r="O67" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C68" s="8"/>
       <c r="D68" s="3" t="str">
@@ -3543,22 +3643,22 @@
         <v>85</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F68" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H68" s="8"/>
       <c r="I68" s="8" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="J68" s="8"/>
       <c r="K68" s="8"/>
       <c r="L68" s="8" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="M68" s="8"/>
       <c r="N68" s="8"/>
@@ -3566,7 +3666,7 @@
     </row>
     <row r="69" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C69" s="8"/>
       <c r="D69" s="3" t="str">
@@ -3574,22 +3674,22 @@
         <v>86</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H69" s="8"/>
       <c r="I69" s="8" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="J69" s="8"/>
       <c r="K69" s="8"/>
       <c r="L69" s="8" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="M69" s="8"/>
       <c r="N69" s="8"/>
@@ -3597,198 +3697,48 @@
     </row>
     <row r="70" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="7"/>
         <v>87</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F70" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G70" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H70" s="8"/>
       <c r="I70" s="8" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="J70" s="8"/>
       <c r="K70" s="8"/>
       <c r="L70" s="8" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="M70" s="8"/>
       <c r="N70" s="8"/>
       <c r="O70" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="183">
-    <mergeCell ref="L69:O69"/>
-    <mergeCell ref="L70:O70"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C45:C50"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="F61:H61"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="G56:H56"/>
+  <mergeCells count="152">
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="C51:C56"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="C57:C60"/>
+    <mergeCell ref="O12:O15"/>
+    <mergeCell ref="O32:O35"/>
+    <mergeCell ref="O37:O39"/>
     <mergeCell ref="I53:K53"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="I65:K65"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="C63:C69"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="L11:L35"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
     <mergeCell ref="C41:C42"/>
     <mergeCell ref="N61:O61"/>
     <mergeCell ref="L62:O62"/>
@@ -3813,6 +3763,125 @@
     <mergeCell ref="I44:K44"/>
     <mergeCell ref="I43:K43"/>
     <mergeCell ref="C43:C44"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="I66:K66"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="L11:L35"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="O16:O23"/>
+    <mergeCell ref="O24:O31"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I70:K70"/>
+    <mergeCell ref="I67:K67"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="I64:K64"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I68:K68"/>
+    <mergeCell ref="C63:C69"/>
+    <mergeCell ref="L69:O69"/>
+    <mergeCell ref="L70:O70"/>
+    <mergeCell ref="C45:C50"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="I65:K65"/>
+    <mergeCell ref="G68:H68"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>